<commit_message>
Publish data update from dashboard
</commit_message>
<xml_diff>
--- a/data/team-data.xlsx
+++ b/data/team-data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\rana.moselhy\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eslamsaad/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7221121C-EA4E-40F3-AD5F-937C409082B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B72ADE9A-0CEA-2545-993A-6F3F8FB1D4B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1140" yWindow="1140" windowWidth="14420" windowHeight="7400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="113">
   <si>
     <t>ID</t>
   </si>
@@ -361,6 +361,9 @@
   </si>
   <si>
     <t>Expert</t>
+  </si>
+  <si>
+    <t>Eslam</t>
   </si>
 </sst>
 </file>
@@ -1064,12 +1067,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:CF6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="84" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:84" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1323,7 +1326,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:84" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1458,7 +1461,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="3" spans="1:84" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1596,7 +1599,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="4" spans="1:84" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1620,7 +1623,7 @@
         <v>85</v>
       </c>
       <c r="L4" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="BA4" t="s">
         <v>97</v>
@@ -1716,7 +1719,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="5" spans="1:84" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1854,7 +1857,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="6" spans="1:84" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:84" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>

</xml_diff>